<commit_message>
Generate input workbooks from a description
solver/scaffold.py writes a template from classes plus split counts, peer classes,
topics and a week range: Groups and Peers prefilled, Calendar as a class x week grid,
Settings and a Read me sheet. One example trip per tutored class is marked so the
template can be planned right away, and the week columns can be headed with Mondays
instead of week numbers, which stays correct across a year change.

main.py --new exposes it; --classes 6a:2 6b:2, --peer-classes, --topics, --weeks.

The calendar header is now matched strictly (36, W36, KW36 or a date), because the
loose scan read week numbers out of the class names of a template whose trip cells
were still blank. A workbook whose groups all come from one class is rejected with
an explanation: the room only opens while a tutored class travels, so that class is
away in every week the room is free.
</commit_message>
<xml_diff>
--- a/example/input.xlsx
+++ b/example/input.xlsx
@@ -454,7 +454,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -884,16 +884,16 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1099,7 +1099,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1120,10 +1120,8 @@
           <t>Max sessions per peer</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B2" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -1132,10 +1130,8 @@
           <t>Max sessions per group per week</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B3" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -1161,7 +1157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -1178,7 +1174,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Groups: one row per class split, plus the class it belongs to.</t>
+          <t>Groups: one row per class split, plus the class it belongs to. Already filled in.</t>
         </is>
       </c>
     </row>
@@ -1220,107 +1216,114 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Calendar: rows are classes, columns are weeks; an x marks a class trip. Please list</t>
+          <t>Calendar: rows are classes, columns are weeks; an x marks a class trip. Both the</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>both the tutored classes and the classes the peers come from.</t>
+          <t>tutored classes and the peer classes are listed - please keep them, the planner</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Settings: optional. 'Max sessions per peer' is the default limit for peers that</t>
+          <t>reads both.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>leave their own limit blank; 'Max sessions per group per week' caps how many</t>
+          <t>Settings: 'Max sessions per peer' is the default limit for peers that leave their</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>sessions one class group may have in the same week (blank = no cap); 'Blackout</t>
+          <t>own limit blank; 'Max sessions per group per week' caps how many sessions one class</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>weeks' are weeks with no mentoring at all (holidays, exam weeks, project weeks).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15"/>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>The rules:</t>
-        </is>
-      </c>
-    </row>
+          <t>group may have in the same week (blank = no cap); 'Blackout weeks' are weeks with no</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>mentoring at all (holidays, exam weeks, project weeks).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  A room exists only in weeks where a TUTORED class is on a trip - a trip of a</t>
+          <t>The rules:</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  peer's class does not open a room, it only makes that peer unavailable.</t>
+          <t xml:space="preserve">  A room exists only in weeks where a TUTORED class is on a trip - a trip of a</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  A group never meets in a week when its own class is away; a peer group never meets</t>
+          <t xml:space="preserve">  peer's class does not open a room, it only makes that peer unavailable.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  in a week when any of its pupils' classes is away.</t>
+          <t xml:space="preserve">  A group never meets in a week when its own class is away; a peer group never meets</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Every group does every topic exactly once, so it has one session per topic. A</t>
+          <t xml:space="preserve">  in a week when any of its pupils' classes is away.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Every group does every topic exactly once, so it has one session per topic. A</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t xml:space="preserve">  week may hold several sessions for one group; the planner spreads them where it can.</t>
         </is>
       </c>
     </row>
-    <row r="23"/>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Run: uv run python main.py example/input.xlsx</t>
-        </is>
-      </c>
-    </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>The sheets Plan, Sessions, Loads, Overview and Notes are written for you.</t>
+          <t>Fill in the peer surnames and the trips, then run the planner. The sheets Plan,</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Sessions, Loads, Overview and Notes are written for you.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Serve the planner in a browser window
solver/app.py serves one page with two cards: upload a workbook and get it back
planned, or create a new one - classes with split counts, peer classes, topics, a
date for the first week, then a class x week grid to tick the trips in and the
limits to set. It is stdlib only (http.server on 127.0.0.1) so the bundled exe
stays small, and the pages live in solver/static.

main.py --app (with --port, --no-browser) starts it; a bundled exe with no
arguments starts it by itself, and its default workbook is the one next to the exe.
</commit_message>
<xml_diff>
--- a/example/input.xlsx
+++ b/example/input.xlsx
@@ -1157,7 +1157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -1230,100 +1230,121 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>reads both.</t>
+          <t>reads both. The template starts with one example trip per tutored class, each in a</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Settings: 'Max sessions per peer' is the default limit for peers that leave their</t>
+          <t>different week, so it can be planned right away - replace them with the real ones.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>own limit blank; 'Max sessions per group per week' caps how many sessions one class</t>
+          <t>Settings: 'Max sessions per peer' is the default limit for peers that leave their</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>group may have in the same week (blank = no cap); 'Blackout weeks' are weeks with no</t>
+          <t>own limit blank; 'Max sessions per group per week' caps how many sessions one class</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>group may have in the same week (blank = no cap); 'Blackout weeks' are weeks with no</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>mentoring at all (holidays, exam weeks, project weeks).</t>
         </is>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>The rules:</t>
-        </is>
-      </c>
-    </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  A room exists only in weeks where a TUTORED class is on a trip - a trip of a</t>
+          <t>The rules:</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  peer's class does not open a room, it only makes that peer unavailable.</t>
+          <t xml:space="preserve">  A room exists only in weeks where a TUTORED class is on a trip - a trip of a</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  A group never meets in a week when its own class is away; a peer group never meets</t>
+          <t xml:space="preserve">  peer's class does not open a room, it only makes that peer unavailable.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  in a week when any of its pupils' classes is away.</t>
+          <t xml:space="preserve">  A group never meets in a week when its own class is away; a peer group never meets</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Every group does every topic exactly once, so it has one session per topic. A</t>
+          <t xml:space="preserve">  in a week when any of its pupils' classes is away.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Every group does every topic exactly once, so it has one session per topic. A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t xml:space="preserve">  week may hold several sessions for one group; the planner spreads them where it can.</t>
         </is>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Fill in the peer surnames and the trips, then run the planner. The sheets Plan,</t>
-        </is>
-      </c>
-    </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Sessions, Loads, Overview and Notes are written for you.</t>
+          <t>Fill in the peer surnames and the trips, then run the planner: double click</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>mentoring-planner.exe and a window opens where you pick this file, or run</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>'python main.py &lt;this file&gt;' in a shell. The sheets Plan, Sessions, Loads, Overview</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>and Notes are written for you - they are replaced on every run.</t>
         </is>
       </c>
     </row>

</xml_diff>